<commit_message>
Case-insensitive Parent grouping: merge casing-only duplicates (215->211 diseases)
Merges 'Multiple sclerosis'/'Multiple Sclerosis' and 3 other casing-only Parent
duplicates (Eosinophilic Esophagitis, Inclusion Body Myositis, Rheumatic Chorea).
Rebuilds all reports (1-7) and DOID/SNOMED Gilda grounding CSVs at 211 diseases.
README updated with final counts and method notes.
</commit_message>
<xml_diff>
--- a/data/4-reports/2_Proposed_Diseases.xlsx
+++ b/data/4-reports/2_Proposed_Diseases.xlsx
@@ -1908,7 +1908,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001106</t>
+          <t>ARI:0001105</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001154</t>
+          <t>ARI:0001151</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Remove generic 'Autoimmune disease' group entry (210 diseases)
Excludes the master 'Autoimmune disease' parent (syn=G, Category All) as too generic;
'Myocarditis due to autoimmune disease' (a specific disease) is retained. Rebuilds all
reports (1-7) and DOID/SNOMED grounding CSVs at 210 diseases. README updated.
</commit_message>
<xml_diff>
--- a/data/4-reports/2_Proposed_Diseases.xlsx
+++ b/data/4-reports/2_Proposed_Diseases.xlsx
@@ -1313,7 +1313,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001034</t>
+          <t>ARI:0001033</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001035</t>
+          <t>ARI:0001034</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001072</t>
+          <t>ARI:0001071</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001075</t>
+          <t>ARI:0001074</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001105</t>
+          <t>ARI:0001104</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001151</t>
+          <t>ARI:0001150</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">

</xml_diff>